<commit_message>
Play payload decision screens side by side and open lessons 7–9 from the map.
Sheet cash, jumps, and conditional copy stay intact, and Lesson 8 choices use the spotlight layout.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/Screens1.xlsx
+++ b/lib/academy/lessons/payload/source/Screens1.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="428">
   <si>
     <t>Module Number</t>
   </si>
@@ -1178,16 +1178,13 @@
     <t>Slide until $18 is set aside for the cinema. $12 stays in the jar.</t>
   </si>
   <si>
-    <t>Lars remembers he still needs to pay for Senna's headphones that he broke.
-Replacing Senna's headphones is a...</t>
-  </si>
-  <si>
-    <t>Holly remembers she still needs to pay for Mia's headphones that she broke.
-Replacing Mia's headphones is a...</t>
-  </si>
-  <si>
-    <t>Aiden remembers he still needs to pay for Dash's headphones that he broke.
-Replacing Dash's headphones is a...</t>
+    <t>Lars remembers he still needs to pay for Senna's headphones that he broke. Replacing Senna's headphones is a...</t>
+  </si>
+  <si>
+    <t>Holly remembers she still needs to pay for Mia's headphones that she broke. Replacing Mia's headphones is a...</t>
+  </si>
+  <si>
+    <t>Aiden remembers he still needs to pay for Dash's headphones that he broke. Replacing Dash's headphones is a...</t>
   </si>
   <si>
     <t>savings-goal</t>
@@ -1536,14 +1533,22 @@
     <t>CHOICE A: Want CHOICE B: Need CORRECT: B</t>
   </si>
   <si>
-    <t>IF cash &gt;= 8 THEN CHOICE A: Pay $8 → SET cash=cash-8 → GO Screen 3
-ELSE show button “See what would have happened if she hadn’t bought the case” → GO Screen 2-alt
-CHOICE B: Can’t cover it → GO Screen 3</t>
-  </si>
-  <si>
-    <t>IF cash &gt;= 8 THEN CHOICE A: Pay $8 → SET cash=cash-8 → GO Screen 3
-ELSE show button “See what would have happened if he hadn’t bought the case” → GO Screen 2-alt
-CHOICE B: Can’t cover it → GO Screen 3</t>
+    <t>IF cash &gt;= 8 THEN
+CHOICE A: Pay $8 → SET cash=cash-8 → GO Screen 3
+CHOICE B: Can’t cover it → GO Screen 3
+IF cash &lt; 8 THEN
+TEXT: Holly has {cash} left. The arcade card is $8, so she can’t pay. What do you want Holly to do?
+CHOICE A: See what would have happened if she hadn’t bought the case → GO Screen 2-alt
+CHOICE B: Skip the arcade → GO Screen 3</t>
+  </si>
+  <si>
+    <t>IF cash &gt;= 8 THEN
+CHOICE A: Pay $8 → SET cash=cash-8 → GO Screen 3
+CHOICE B: Can’t cover it → GO Screen 3
+IF cash &lt; 8 THEN
+TEXT: Lars has {cash} left. The arcade card is $8, so he can’t pay. What do you want Lars to do?
+CHOICE A: See what would have happened if he hadn’t bought the case → GO Screen 2-alt
+CHOICE B: Skip the arcade → GO Screen 3</t>
   </si>
   <si>
     <t>MEDAL: bronze</t>
@@ -1676,6 +1681,45 @@
   </si>
   <si>
     <t>OPTIONS: afford | want | see CORRECT: afford</t>
+  </si>
+  <si>
+    <t>Replacing Senna's headphones comes before the gelato. Which skill is that?</t>
+  </si>
+  <si>
+    <t>Replacing Mia's headphones comes before the gelato. Which skill is that?</t>
+  </si>
+  <si>
+    <t>Replacing Dash's headphones comes before the energy drink. Which skill is that?</t>
+  </si>
+  <si>
+    <t>CHOICE A: Stop &amp; Think CHOICE B: Put Needs First CHOICE C: Keep Spare Cash CORRECT: B</t>
+  </si>
+  <si>
+    <t>That skill is Put Needs First.</t>
+  </si>
+  <si>
+    <t>Sharing the gelato leaves Lars some money. Buying his own leaves $0. Which skill is he using when he shares?</t>
+  </si>
+  <si>
+    <t>Sharing the gelato leaves Holly some money. Buying her own leaves $0. Which skill is she using when she shares?</t>
+  </si>
+  <si>
+    <t>Splitting the 2-for-1 energy drink leaves Aiden some money. Buying one at full price leaves $0. Which skill is he using?</t>
+  </si>
+  <si>
+    <t>CHOICE A: Stop &amp; Think CHOICE B: Put Needs First CHOICE C: Keep Spare Cash CORRECT: C</t>
+  </si>
+  <si>
+    <t>That skill is Keep Spare Cash.</t>
+  </si>
+  <si>
+    <t>IF cash &gt;= 8 THEN
+CHOICE A: Pay $8 → SET cash=cash-8 → GO Screen 3
+CHOICE B: Can’t cover it → GO Screen 3
+IF cash &lt; 8 THEN
+TEXT: Aiden has {cash} left. The arcade card is $8, so he can’t pay. What do you want Aiden to do?
+CHOICE A: See what would have happened if he hadn’t bought the case → GO Screen 2-alt
+CHOICE B: Skip the arcade → GO Screen 3</t>
   </si>
 </sst>
 </file>
@@ -2066,7 +2110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" style="1" customWidth="1"/>
@@ -4143,7 +4187,7 @@
         <v>7</v>
       </c>
       <c r="C51" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>274</v>
@@ -4194,7 +4238,7 @@
         <v>7</v>
       </c>
       <c r="C52" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>277</v>
@@ -4244,7 +4288,7 @@
         <v>7</v>
       </c>
       <c r="C53" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>279</v>
@@ -4295,7 +4339,7 @@
         <v>7</v>
       </c>
       <c r="C54" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>284</v>
@@ -4324,7 +4368,7 @@
         <v>1</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>351</v>
@@ -4374,7 +4418,7 @@
         <v>2</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>365</v>
@@ -4401,7 +4445,7 @@
         <v>383</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>384</v>
+        <v>427</v>
       </c>
     </row>
     <row r="57" spans="1:17" ht="32" x14ac:dyDescent="0.2">
@@ -4456,7 +4500,7 @@
         <v>3</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>330</v>
@@ -4579,7 +4623,7 @@
         <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>334</v>
@@ -4620,7 +4664,7 @@
         <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>302</v>
@@ -5073,6 +5117,106 @@
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
+    </row>
+    <row r="76" spans="1:17">
+      <c r="A76" s="1">
+        <v>1</v>
+      </c>
+      <c r="B76" s="1">
+        <v>7</v>
+      </c>
+      <c r="C76" s="1">
+        <v>3</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="O76" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="P76" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17">
+      <c r="A77" s="1">
+        <v>1</v>
+      </c>
+      <c r="B77" s="1">
+        <v>7</v>
+      </c>
+      <c r="C77" s="1">
+        <v>6</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="M77" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="N77" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="O77" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="P77" s="2" t="s">
+        <v>426</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q73" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>